<commit_message>
new version works perfectly
</commit_message>
<xml_diff>
--- a/GMC_failed_to_download.xlsx
+++ b/GMC_failed_to_download.xlsx
@@ -556,1298 +556,928 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>586969770</t>
-        </is>
+      <c r="A26" t="n">
+        <v>586969770</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>587300945</t>
-        </is>
+      <c r="A27" t="n">
+        <v>587300945</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>28635034</t>
-        </is>
+      <c r="A28" t="n">
+        <v>28635034</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>587091464</t>
-        </is>
+      <c r="A29" t="n">
+        <v>587091464</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>587245314</t>
-        </is>
+      <c r="A30" t="n">
+        <v>587245314</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>586694475</t>
-        </is>
+      <c r="A31" t="n">
+        <v>586694475</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>586995106</t>
-        </is>
+      <c r="A32" t="n">
+        <v>586995106</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>28420341</t>
-        </is>
+      <c r="A33" t="n">
+        <v>28420341</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>586769242</t>
-        </is>
+      <c r="A34" t="n">
+        <v>586769242</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>587274062</t>
-        </is>
+      <c r="A35" t="n">
+        <v>587274062</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>587358646</t>
-        </is>
+      <c r="A36" t="n">
+        <v>587358646</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>586334008</t>
-        </is>
+      <c r="A37" t="n">
+        <v>586334008</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>586708852</t>
-        </is>
+      <c r="A38" t="n">
+        <v>586708852</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>586778144</t>
-        </is>
+      <c r="A39" t="n">
+        <v>586778144</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>586730993</t>
-        </is>
+      <c r="A40" t="n">
+        <v>586730993</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>28607151</t>
-        </is>
+      <c r="A41" t="n">
+        <v>28607151</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>587047386</t>
-        </is>
+      <c r="A42" t="n">
+        <v>587047386</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>586832200</t>
-        </is>
+      <c r="A43" t="n">
+        <v>586832200</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>587068698</t>
-        </is>
+      <c r="A44" t="n">
+        <v>587068698</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>586633970</t>
-        </is>
+      <c r="A45" t="n">
+        <v>586633970</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>587093117</t>
-        </is>
+      <c r="A46" t="n">
+        <v>587093117</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>586992176</t>
-        </is>
+      <c r="A47" t="n">
+        <v>586992176</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>28520897</t>
-        </is>
+      <c r="A48" t="n">
+        <v>28520897</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>28395075</t>
-        </is>
+      <c r="A49" t="n">
+        <v>28395075</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>586972585</t>
-        </is>
+      <c r="A50" t="n">
+        <v>586972585</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>28605690</t>
-        </is>
+      <c r="A51" t="n">
+        <v>28605690</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>586776639</t>
-        </is>
+      <c r="A52" t="n">
+        <v>586776639</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>586693165</t>
-        </is>
+      <c r="A53" t="n">
+        <v>586693165</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>28349330</t>
-        </is>
+      <c r="A54" t="n">
+        <v>28349330</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>587029785</t>
-        </is>
+      <c r="A55" t="n">
+        <v>587029785</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>586513129</t>
-        </is>
+      <c r="A56" t="n">
+        <v>586513129</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>28606648</t>
-        </is>
+      <c r="A57" t="n">
+        <v>28606648</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>586512992</t>
-        </is>
+      <c r="A58" t="n">
+        <v>586512992</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>587049670</t>
-        </is>
+      <c r="A59" t="n">
+        <v>587049670</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>586526720</t>
-        </is>
+      <c r="A60" t="n">
+        <v>586526720</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>28705519</t>
-        </is>
+      <c r="A61" t="n">
+        <v>28705519</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>586992632</t>
-        </is>
+      <c r="A62" t="n">
+        <v>586992632</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>587048005</t>
-        </is>
+      <c r="A63" t="n">
+        <v>587048005</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>586516917</t>
-        </is>
+      <c r="A64" t="n">
+        <v>586516917</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>28622836</t>
-        </is>
+      <c r="A65" t="n">
+        <v>28622836</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>586792327</t>
-        </is>
+      <c r="A66" t="n">
+        <v>586792327</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>586583251</t>
-        </is>
+      <c r="A67" t="n">
+        <v>586583251</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>28307234</t>
-        </is>
+      <c r="A68" t="n">
+        <v>28307234</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>586505724</t>
-        </is>
+      <c r="A69" t="n">
+        <v>586505724</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>586522165</t>
-        </is>
+      <c r="A70" t="n">
+        <v>586522165</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>587046042</t>
-        </is>
+      <c r="A71" t="n">
+        <v>587046042</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>586881317</t>
-        </is>
+      <c r="A72" t="n">
+        <v>586881317</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>587184214</t>
-        </is>
+      <c r="A73" t="n">
+        <v>587184214</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>586736968</t>
-        </is>
+      <c r="A74" t="n">
+        <v>586736968</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>586414162</t>
-        </is>
+      <c r="A75" t="n">
+        <v>586414162</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>28425358</t>
-        </is>
+      <c r="A76" t="n">
+        <v>28425358</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>587021926</t>
-        </is>
+      <c r="A77" t="n">
+        <v>587021926</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>586990320</t>
-        </is>
+      <c r="A78" t="n">
+        <v>586990320</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>586822392</t>
-        </is>
+      <c r="A79" t="n">
+        <v>586822392</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>586350429</t>
-        </is>
+      <c r="A80" t="n">
+        <v>586350429</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>28298990</t>
-        </is>
+      <c r="A81" t="n">
+        <v>28298990</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>587052852</t>
-        </is>
+      <c r="A82" t="n">
+        <v>587052852</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>586994920</t>
-        </is>
+      <c r="A83" t="n">
+        <v>586994920</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>586326092</t>
-        </is>
+      <c r="A84" t="n">
+        <v>586326092</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>587030188</t>
-        </is>
+      <c r="A85" t="n">
+        <v>587030188</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>586991648</t>
-        </is>
+      <c r="A86" t="n">
+        <v>586991648</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>587080969</t>
-        </is>
+      <c r="A87" t="n">
+        <v>587080969</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>587180233</t>
-        </is>
+      <c r="A88" t="n">
+        <v>587180233</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>28653762</t>
-        </is>
+      <c r="A89" t="n">
+        <v>28653762</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>587052957</t>
-        </is>
+      <c r="A90" t="n">
+        <v>587052957</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>587151480</t>
-        </is>
+      <c r="A91" t="n">
+        <v>587151480</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>587047230</t>
-        </is>
+      <c r="A92" t="n">
+        <v>587047230</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>28286587</t>
-        </is>
+      <c r="A93" t="n">
+        <v>28286587</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>587261772</t>
-        </is>
+      <c r="A94" t="n">
+        <v>587261772</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>587262120</t>
-        </is>
+      <c r="A95" t="n">
+        <v>587262120</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>586983851</t>
-        </is>
+      <c r="A96" t="n">
+        <v>586983851</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>587043614</t>
-        </is>
+      <c r="A97" t="n">
+        <v>587043614</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>587007450</t>
-        </is>
+      <c r="A98" t="n">
+        <v>587007450</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>586711818</t>
-        </is>
+      <c r="A99" t="n">
+        <v>586711818</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>28425153</t>
-        </is>
+      <c r="A100" t="n">
+        <v>28425153</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>587251543</t>
-        </is>
+      <c r="A101" t="n">
+        <v>587251543</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>587066749</t>
-        </is>
+      <c r="A102" t="n">
+        <v>587066749</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>28572648</t>
-        </is>
+      <c r="A103" t="n">
+        <v>28572648</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>28309628</t>
-        </is>
+      <c r="A104" t="n">
+        <v>28309628</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>586708741</t>
-        </is>
+      <c r="A105" t="n">
+        <v>586708741</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>587150423</t>
-        </is>
+      <c r="A106" t="n">
+        <v>587150423</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>28496562</t>
-        </is>
+      <c r="A107" t="n">
+        <v>28496562</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>586959601</t>
-        </is>
+      <c r="A108" t="n">
+        <v>586959601</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>587277643</t>
-        </is>
+      <c r="A109" t="n">
+        <v>587277643</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>586986283</t>
-        </is>
+      <c r="A110" t="n">
+        <v>586986283</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>587019468</t>
-        </is>
+      <c r="A111" t="n">
+        <v>587019468</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>28635802</t>
-        </is>
+      <c r="A112" t="n">
+        <v>28635802</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>586377292</t>
-        </is>
+      <c r="A113" t="n">
+        <v>586377292</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>587183657</t>
-        </is>
+      <c r="A114" t="n">
+        <v>587183657</v>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>586869659</t>
-        </is>
+      <c r="A115" t="n">
+        <v>586869659</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>587090155</t>
-        </is>
+      <c r="A116" t="n">
+        <v>587090155</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>586417076</t>
-        </is>
+      <c r="A117" t="n">
+        <v>586417076</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>586466884</t>
-        </is>
+      <c r="A118" t="n">
+        <v>586466884</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>28281127</t>
-        </is>
+      <c r="A119" t="n">
+        <v>28281127</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>28424954</t>
-        </is>
+      <c r="A120" t="n">
+        <v>28424954</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>586710210</t>
-        </is>
+      <c r="A121" t="n">
+        <v>586710210</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>586425345</t>
-        </is>
+      <c r="A122" t="n">
+        <v>586425345</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>586956492</t>
-        </is>
+      <c r="A123" t="n">
+        <v>586956492</v>
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>587154934</t>
-        </is>
+      <c r="A124" t="n">
+        <v>587154934</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>586499106</t>
-        </is>
+      <c r="A125" t="n">
+        <v>586499106</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>587010055</t>
-        </is>
+      <c r="A126" t="n">
+        <v>587010055</v>
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>587094127</t>
-        </is>
+      <c r="A127" t="n">
+        <v>587094127</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>28423322</t>
-        </is>
+      <c r="A128" t="n">
+        <v>28423322</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>586508652</t>
-        </is>
+      <c r="A129" t="n">
+        <v>586508652</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>587045324</t>
-        </is>
+      <c r="A130" t="n">
+        <v>587045324</v>
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>587066834</t>
-        </is>
+      <c r="A131" t="n">
+        <v>587066834</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>586852162</t>
-        </is>
+      <c r="A132" t="n">
+        <v>586852162</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>587064571</t>
-        </is>
+      <c r="A133" t="n">
+        <v>587064571</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>587183306</t>
-        </is>
+      <c r="A134" t="n">
+        <v>587183306</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>28623768</t>
-        </is>
+      <c r="A135" t="n">
+        <v>28623768</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>586706143</t>
-        </is>
+      <c r="A136" t="n">
+        <v>586706143</v>
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>587087460</t>
-        </is>
+      <c r="A137" t="n">
+        <v>587087460</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>28492871</t>
-        </is>
+      <c r="A138" t="n">
+        <v>28492871</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>586492181</t>
-        </is>
+      <c r="A139" t="n">
+        <v>586492181</v>
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>587159639</t>
-        </is>
+      <c r="A140" t="n">
+        <v>587159639</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>586591799</t>
-        </is>
+      <c r="A141" t="n">
+        <v>586591799</v>
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>586693591</t>
-        </is>
+      <c r="A142" t="n">
+        <v>586693591</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>586995119</t>
-        </is>
+      <c r="A143" t="n">
+        <v>586995119</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>586414619</t>
-        </is>
+      <c r="A144" t="n">
+        <v>586414619</v>
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>586866441</t>
-        </is>
+      <c r="A145" t="n">
+        <v>586866441</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>586703294</t>
-        </is>
+      <c r="A146" t="n">
+        <v>586703294</v>
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>586624617</t>
-        </is>
+      <c r="A147" t="n">
+        <v>586624617</v>
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>586986323</t>
-        </is>
+      <c r="A148" t="n">
+        <v>586986323</v>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>28373356</t>
-        </is>
+      <c r="A149" t="n">
+        <v>28373356</v>
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>586739521</t>
-        </is>
+      <c r="A150" t="n">
+        <v>586739521</v>
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>587017195</t>
-        </is>
+      <c r="A151" t="n">
+        <v>587017195</v>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>587094541</t>
-        </is>
+      <c r="A152" t="n">
+        <v>587094541</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>586494121</t>
-        </is>
+      <c r="A153" t="n">
+        <v>586494121</v>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>587251051</t>
-        </is>
+      <c r="A154" t="n">
+        <v>587251051</v>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>587080402</t>
-        </is>
+      <c r="A155" t="n">
+        <v>587080402</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>586709545</t>
-        </is>
+      <c r="A156" t="n">
+        <v>586709545</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>587098828</t>
-        </is>
+      <c r="A157" t="n">
+        <v>587098828</v>
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>587009747</t>
-        </is>
+      <c r="A158" t="n">
+        <v>587009747</v>
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>587116838</t>
-        </is>
+      <c r="A159" t="n">
+        <v>587116838</v>
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>586983117</t>
-        </is>
+      <c r="A160" t="n">
+        <v>586983117</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>586304540</t>
-        </is>
+      <c r="A161" t="n">
+        <v>586304540</v>
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>587183880</t>
-        </is>
+      <c r="A162" t="n">
+        <v>587183880</v>
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>586579070</t>
-        </is>
+      <c r="A163" t="n">
+        <v>586579070</v>
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>587244986</t>
-        </is>
+      <c r="A164" t="n">
+        <v>587244986</v>
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>586848900</t>
-        </is>
+      <c r="A165" t="n">
+        <v>586848900</v>
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>586271475</t>
-        </is>
+      <c r="A166" t="n">
+        <v>586271475</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>587016371</t>
-        </is>
+      <c r="A167" t="n">
+        <v>587016371</v>
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>587072067</t>
-        </is>
+      <c r="A168" t="n">
+        <v>587072067</v>
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>587150111</t>
-        </is>
+      <c r="A169" t="n">
+        <v>587150111</v>
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>587163384</t>
-        </is>
+      <c r="A170" t="n">
+        <v>587163384</v>
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>586998506</t>
-        </is>
+      <c r="A171" t="n">
+        <v>586998506</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>586403206</t>
-        </is>
+      <c r="A172" t="n">
+        <v>586403206</v>
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>28498730</t>
-        </is>
+      <c r="A173" t="n">
+        <v>28498730</v>
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>28419233</t>
-        </is>
+      <c r="A174" t="n">
+        <v>28419233</v>
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>587048283</t>
-        </is>
+      <c r="A175" t="n">
+        <v>587048283</v>
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>28498193</t>
-        </is>
+      <c r="A176" t="n">
+        <v>28498193</v>
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>586305533</t>
-        </is>
+      <c r="A177" t="n">
+        <v>586305533</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>586820544</t>
-        </is>
+      <c r="A178" t="n">
+        <v>586820544</v>
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>586650437</t>
-        </is>
+      <c r="A179" t="n">
+        <v>586650437</v>
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>28698670</t>
-        </is>
+      <c r="A180" t="n">
+        <v>28698670</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>586356881</t>
-        </is>
+      <c r="A181" t="n">
+        <v>586356881</v>
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>28502724</t>
-        </is>
+      <c r="A182" t="n">
+        <v>28502724</v>
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>587249350</t>
-        </is>
+      <c r="A183" t="n">
+        <v>587249350</v>
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>587069436</t>
-        </is>
+      <c r="A184" t="n">
+        <v>587069436</v>
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>28489707</t>
-        </is>
+      <c r="A185" t="n">
+        <v>28489707</v>
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>28696984</t>
-        </is>
+      <c r="A186" t="n">
+        <v>28696984</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>586287796</t>
-        </is>
+      <c r="A187" t="n">
+        <v>586287796</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>28085773</t>
-        </is>
+      <c r="A188" t="n">
+        <v>28085773</v>
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>28631316</t>
-        </is>
+      <c r="A189" t="n">
+        <v>28631316</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>586993422</t>
-        </is>
+      <c r="A190" t="n">
+        <v>586993422</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>587045866</t>
-        </is>
+      <c r="A191" t="n">
+        <v>587045866</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>587220397</t>
-        </is>
+      <c r="A192" t="n">
+        <v>587220397</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>586409841</t>
-        </is>
+      <c r="A193" t="n">
+        <v>586409841</v>
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>586994925</t>
-        </is>
+      <c r="A194" t="n">
+        <v>586994925</v>
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>587138502</t>
-        </is>
+      <c r="A195" t="n">
+        <v>587138502</v>
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>587302205</t>
-        </is>
+      <c r="A196" t="n">
+        <v>587302205</v>
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>28283139</t>
-        </is>
+      <c r="A197" t="n">
+        <v>28283139</v>
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>586879965</t>
-        </is>
+      <c r="A198" t="n">
+        <v>586879965</v>
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>586578443</t>
-        </is>
+      <c r="A199" t="n">
+        <v>586578443</v>
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>587071139</t>
-        </is>
+      <c r="A200" t="n">
+        <v>587071139</v>
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>586985471</t>
-        </is>
+      <c r="A201" t="n">
+        <v>586985471</v>
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>587180223</t>
-        </is>
+      <c r="A202" t="n">
+        <v>587180223</v>
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>587042870</t>
-        </is>
+      <c r="A203" t="n">
+        <v>587042870</v>
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>28133584</t>
-        </is>
+      <c r="A204" t="n">
+        <v>28133584</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>28299072</t>
-        </is>
+      <c r="A205" t="n">
+        <v>28299072</v>
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>28349205</t>
-        </is>
+      <c r="A206" t="n">
+        <v>28349205</v>
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>587051212</t>
-        </is>
+      <c r="A207" t="n">
+        <v>587051212</v>
       </c>
     </row>
     <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>586873222</t>
-        </is>
+      <c r="A208" t="n">
+        <v>586873222</v>
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>586966482</t>
-        </is>
+      <c r="A209" t="n">
+        <v>586966482</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>587065548</t>
-        </is>
+      <c r="A210" t="n">
+        <v>587065548</v>
       </c>
     </row>
   </sheetData>

</xml_diff>